<commit_message>
se avanza con el back, se modifica controller, service y model del sacs para poder llamar ubicacion de la DB neon
</commit_message>
<xml_diff>
--- a/src/main/resources/reports/reporte_rms_vss_cctv.xlsx
+++ b/src/main/resources/reports/reporte_rms_vss_cctv.xlsx
@@ -55,7 +55,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1130" uniqueCount="108">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1141" uniqueCount="117">
   <si>
     <t>Registro de Mantenimiento Sistema VSS</t>
   </si>
@@ -379,6 +379,33 @@
   </si>
   <si>
     <t xml:space="preserve">ASCENSOR PANORAMICO </t>
+  </si>
+  <si>
+    <t>0-16-01</t>
+  </si>
+  <si>
+    <t>FASE 1</t>
+  </si>
+  <si>
+    <t>CARCAMO BHS</t>
+  </si>
+  <si>
+    <t>3-48-1</t>
+  </si>
+  <si>
+    <t>RAMPA PUENTE 89</t>
+  </si>
+  <si>
+    <t>20/03/2026</t>
+  </si>
+  <si>
+    <t>2-43-7</t>
+  </si>
+  <si>
+    <t>PUENTE 54-55-56</t>
+  </si>
+  <si>
+    <t>21/03/2026</t>
   </si>
 </sst>
 </file>
@@ -5332,9 +5359,15 @@
         <f t="shared" si="1"/>
         <v>8</v>
       </c>
-      <c r="AD20" s="87"/>
-      <c r="AE20" s="76"/>
-      <c r="AF20" s="88"/>
+      <c r="AD20" s="87" t="s">
+        <v>108</v>
+      </c>
+      <c r="AE20" s="76" t="s">
+        <v>109</v>
+      </c>
+      <c r="AF20" s="88" t="s">
+        <v>110</v>
+      </c>
       <c r="AG20" s="77"/>
       <c r="AH20" s="38"/>
       <c r="AI20" s="38"/>
@@ -8774,9 +8807,15 @@
       <c r="B65" s="69">
         <v>1</v>
       </c>
-      <c r="C65" s="79"/>
-      <c r="D65" s="80"/>
-      <c r="E65" s="81"/>
+      <c r="C65" s="79" t="s">
+        <v>111</v>
+      </c>
+      <c r="D65" s="80" t="s">
+        <v>78</v>
+      </c>
+      <c r="E65" s="81" t="s">
+        <v>112</v>
+      </c>
       <c r="F65" s="77"/>
       <c r="G65" s="38">
         <v>1</v>
@@ -8819,9 +8858,15 @@
       <c r="AC65" s="69">
         <v>1</v>
       </c>
-      <c r="AD65" s="110"/>
-      <c r="AE65" s="111"/>
-      <c r="AF65" s="112"/>
+      <c r="AD65" s="110" t="s">
+        <v>114</v>
+      </c>
+      <c r="AE65" s="111" t="s">
+        <v>78</v>
+      </c>
+      <c r="AF65" s="112" t="s">
+        <v>115</v>
+      </c>
       <c r="AG65" s="113">
         <v>0</v>
       </c>
@@ -10046,7 +10091,9 @@
       <c r="M85" s="30"/>
       <c r="N85" s="3"/>
       <c r="O85" s="21"/>
-      <c r="P85" s="41"/>
+      <c r="P85" s="41" t="s">
+        <v>113</v>
+      </c>
       <c r="Q85" s="157"/>
       <c r="R85" s="157"/>
       <c r="S85" s="157"/>
@@ -10070,7 +10117,9 @@
       <c r="AN85" s="30"/>
       <c r="AO85" s="3"/>
       <c r="AP85" s="21"/>
-      <c r="AQ85" s="41"/>
+      <c r="AQ85" s="41" t="s">
+        <v>116</v>
+      </c>
       <c r="AR85" s="157"/>
       <c r="AS85" s="157"/>
       <c r="AT85" s="157"/>

</xml_diff>